<commit_message>
Improve cb torando and whirlpool process
</commit_message>
<xml_diff>
--- a/ssp_modeling/cb/cb_cost_factors/cb_config_params.xlsx
+++ b/ssp_modeling/cb/cb_cost_factors/cb_config_params.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10208"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10302"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fabianfuentes/git/ssp_uganda_data/ssp_modeling/cb/cb_cost_factors/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alexa/Projects/ssp_uganda_data/ssp_modeling/cb/cb_cost_factors/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11EE5FCF-F07C-A645-B65B-E640C083F101}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C7AA21F-1A25-C744-91DF-9CE8EE3F55A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-51200" yWindow="-7160" windowWidth="37680" windowHeight="28200" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17420" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="tx_table" sheetId="1" r:id="rId1"/>
@@ -6387,7 +6387,7 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>

</xml_diff>